<commit_message>
bugfix, v407, scale/degree/0/non <> text
</commit_message>
<xml_diff>
--- a/配對規則.xlsx
+++ b/配對規則.xlsx
@@ -24,11 +24,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -49,7 +50,7 @@
       <sz val="12"/>
       <color rgb="FFFFFF00"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="12"/>
@@ -67,25 +68,25 @@
       <sz val="21"/>
       <color rgb="FF00F4FF"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="18"/>
       <color rgb="FF00F4FF"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="24"/>
       <color rgb="FFFFFF00"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
+      <family val="0"/>
     </font>
     <font>
-      <sz val="13.95"/>
+      <sz val="14"/>
       <color rgb="FFFFFF00"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="21"/>
@@ -101,6 +102,12 @@
     </font>
     <font>
       <sz val="16"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="24"/>
       <color rgb="FFFFFF00"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -159,7 +166,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -246,9 +253,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>762840</xdr:colOff>
+      <xdr:colOff>762480</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>70200</xdr:rowOff>
+      <xdr:rowOff>69840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -262,7 +269,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1694880" y="921600"/>
-          <a:ext cx="6383160" cy="4187880"/>
+          <a:ext cx="6382800" cy="4187520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -328,19 +335,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>654480</xdr:colOff>
+      <xdr:colOff>654120</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>12960</xdr:rowOff>
+      <xdr:rowOff>12600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="3" name="Text Frame 2"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8881560" y="371880"/>
-          <a:ext cx="3965040" cy="1104120"/>
+          <a:ext cx="3964680" cy="1103760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -353,12 +360,22 @@
           <a:round/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="18000" tIns="18000" rIns="18000" bIns="18000" anchor="ctr">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -393,16 +410,17 @@
             <a:t>MIN_DIST ~ MAX_DIST</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -437,16 +455,17 @@
             <a:t>&lt; TOLERANCE_ROT</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -492,16 +511,17 @@
             <a:t>&lt; ORTHO_TOL</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -547,9 +567,6 @@
             <a:t>&lt; ORTHO_TOL</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
@@ -568,9 +585,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>574920</xdr:colOff>
+      <xdr:colOff>574560</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>32040</xdr:rowOff>
+      <xdr:rowOff>31680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -580,13 +597,19 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2864520" y="797040"/>
-          <a:ext cx="5838480" cy="372960"/>
+          <a:ext cx="5838120" cy="372600"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
-          <a:gdLst/>
+          <a:gdLst>
+            <a:gd name="textAreaLeft" fmla="*/ 0 w 5838120"/>
+            <a:gd name="textAreaRight" fmla="*/ 5838480 w 5838120"/>
+            <a:gd name="textAreaTop" fmla="*/ 0 h 372600"/>
+            <a:gd name="textAreaBottom" fmla="*/ 372960 h 372600"/>
+          </a:gdLst>
           <a:ahLst/>
-          <a:rect l="0" t="0" r="r" b="b"/>
+          <a:cxnLst/>
+          <a:rect l="textAreaLeft" t="textAreaTop" r="textAreaRight" b="textAreaBottom"/>
           <a:pathLst>
             <a:path fill="none" w="16218" h="1036">
               <a:moveTo>
@@ -601,6 +624,7 @@
             </a:path>
           </a:pathLst>
         </a:custGeom>
+        <a:noFill/>
         <a:ln w="18360">
           <a:solidFill>
             <a:srgbClr val="FFD8CE"/>
@@ -610,6 +634,12 @@
           <a:tailEnd len="med" type="triangle" w="med"/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
@@ -622,19 +652,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>792720</xdr:colOff>
+      <xdr:colOff>792360</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>127440</xdr:rowOff>
+      <xdr:rowOff>127080</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="5" name="Text Frame 1"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6293880" y="567360"/>
-          <a:ext cx="2626920" cy="210240"/>
+          <a:ext cx="2626560" cy="209880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -644,11 +674,22 @@
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -679,9 +720,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>564840</xdr:colOff>
+      <xdr:colOff>564480</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>32040</xdr:rowOff>
+      <xdr:rowOff>31680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -691,13 +732,19 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3588120" y="1609920"/>
-          <a:ext cx="5104800" cy="1023120"/>
+          <a:ext cx="5104440" cy="1022760"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
-          <a:gdLst/>
+          <a:gdLst>
+            <a:gd name="textAreaLeft" fmla="*/ 0 w 5104440"/>
+            <a:gd name="textAreaRight" fmla="*/ 5104800 w 5104440"/>
+            <a:gd name="textAreaTop" fmla="*/ 0 h 1022760"/>
+            <a:gd name="textAreaBottom" fmla="*/ 1023120 h 1022760"/>
+          </a:gdLst>
           <a:ahLst/>
-          <a:rect l="0" t="0" r="r" b="b"/>
+          <a:cxnLst/>
+          <a:rect l="textAreaLeft" t="textAreaTop" r="textAreaRight" b="textAreaBottom"/>
           <a:pathLst>
             <a:path fill="none" w="14180" h="2842">
               <a:moveTo>
@@ -712,6 +759,7 @@
             </a:path>
           </a:pathLst>
         </a:custGeom>
+        <a:noFill/>
         <a:ln w="18360">
           <a:solidFill>
             <a:srgbClr val="FFD8CE"/>
@@ -721,6 +769,12 @@
           <a:tailEnd len="med" type="triangle" w="med"/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
@@ -733,9 +787,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>248040</xdr:colOff>
+      <xdr:colOff>247680</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>133560</xdr:rowOff>
+      <xdr:rowOff>133200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -745,7 +799,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1199520" y="86040"/>
-          <a:ext cx="12053160" cy="5574600"/>
+          <a:ext cx="12052800" cy="5574240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -820,19 +874,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>405720</xdr:colOff>
+      <xdr:colOff>405360</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>117360</xdr:rowOff>
+      <xdr:rowOff>117000</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="9" name="Text Frame 6"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="11051280" y="5109120"/>
-          <a:ext cx="1546560" cy="210240"/>
+          <a:ext cx="1546200" cy="209880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -842,11 +896,22 @@
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -921,19 +986,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>604440</xdr:colOff>
+      <xdr:colOff>604080</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>28440</xdr:rowOff>
+      <xdr:rowOff>28080</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="11" name="Text Frame 7"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1846440" y="2857680"/>
-          <a:ext cx="1196280" cy="1559880"/>
+          <a:ext cx="1195920" cy="1559520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -948,12 +1013,22 @@
           <a:round/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="18000" tIns="18000" rIns="18000" bIns="18000" anchor="ctr">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -966,16 +1041,17 @@
             <a:t>球標顏色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -999,16 +1075,17 @@
             <a:t>紅色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -1032,16 +1109,17 @@
             <a:t>黃色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -1065,16 +1143,17 @@
             <a:t>綠色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -1098,16 +1177,17 @@
             <a:t>青色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -1131,16 +1211,17 @@
             <a:t>藍色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -1164,16 +1245,17 @@
             <a:t>洋紅色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -1197,9 +1279,6 @@
             <a:t>依背景色</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="FFFF00"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
@@ -1218,9 +1297,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>29</xdr:col>
-      <xdr:colOff>50040</xdr:colOff>
+      <xdr:colOff>49680</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
+      <xdr:rowOff>104040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1230,7 +1309,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="15067080" y="219240"/>
-          <a:ext cx="8554320" cy="5574600"/>
+          <a:ext cx="8553960" cy="5574240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1261,19 +1340,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>219240</xdr:colOff>
+      <xdr:colOff>218880</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>162720</xdr:rowOff>
+      <xdr:rowOff>162360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="13" name="Text Frame 8"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="15427080" y="504000"/>
-          <a:ext cx="2673720" cy="633960"/>
+          <a:ext cx="2673360" cy="633600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1286,12 +1365,22 @@
           <a:round/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="18000" tIns="18000" rIns="18000" bIns="18000" anchor="ctr">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="2000" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -1304,9 +1393,6 @@
             <a:t>配對失敗範例</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="2000" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="00F4FF"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
@@ -1327,7 +1413,7 @@
       <xdr:col>21</xdr:col>
       <xdr:colOff>115200</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>41040</xdr:rowOff>
+      <xdr:rowOff>41400</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -1337,9 +1423,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="15714360" y="1514160"/>
-          <a:ext cx="1469520" cy="640080"/>
+          <a:ext cx="1469520" cy="640440"/>
           <a:chOff x="15714360" y="1514160"/>
-          <a:chExt cx="1469520" cy="640080"/>
+          <a:chExt cx="1469520" cy="640440"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
@@ -1350,7 +1436,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="15714360" y="1514160"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1373,7 +1459,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1382,13 +1472,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1404,7 +1492,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="16277040" y="1524600"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1427,7 +1515,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1436,13 +1528,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>12</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1458,7 +1548,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="15745680" y="2154240"/>
-            <a:ext cx="1438200" cy="0"/>
+            <a:ext cx="1438200" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -1489,9 +1579,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>625680</xdr:colOff>
+      <xdr:colOff>625320</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>85320</xdr:rowOff>
+      <xdr:rowOff>85680</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -1501,9 +1591,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="15693480" y="2520000"/>
-          <a:ext cx="2000880" cy="654120"/>
+          <a:ext cx="2000520" cy="654480"/>
           <a:chOff x="15693480" y="2520000"/>
-          <a:chExt cx="2000880" cy="654120"/>
+          <a:chExt cx="2000520" cy="654480"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
@@ -1514,7 +1604,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="15693480" y="2520000"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1537,7 +1627,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1546,13 +1640,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1568,7 +1660,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="17027280" y="2530440"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1591,7 +1683,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1600,13 +1696,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>12</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1622,7 +1716,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="15817320" y="3174120"/>
-            <a:ext cx="1438200" cy="0"/>
+            <a:ext cx="1438200" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -1653,9 +1747,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>229680</xdr:colOff>
+      <xdr:colOff>229320</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>30960</xdr:rowOff>
+      <xdr:rowOff>30600</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -1665,9 +1759,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="15662160" y="3454560"/>
-          <a:ext cx="1636200" cy="802800"/>
+          <a:ext cx="1635840" cy="802440"/>
           <a:chOff x="15662160" y="3454560"/>
-          <a:chExt cx="1636200" cy="802800"/>
+          <a:chExt cx="1635840" cy="802440"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
@@ -1678,7 +1772,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="15662160" y="3454560"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1701,7 +1795,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1710,13 +1808,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1732,7 +1828,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="16631280" y="3637800"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1755,7 +1851,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1764,13 +1864,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>12</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1786,7 +1884,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="15781680" y="4068360"/>
-            <a:ext cx="1438200" cy="0"/>
+            <a:ext cx="1438200" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -1813,13 +1911,13 @@
       <xdr:col>19</xdr:col>
       <xdr:colOff>103320</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>60840</xdr:rowOff>
+      <xdr:rowOff>61200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>355320</xdr:colOff>
+      <xdr:colOff>354240</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>139320</xdr:rowOff>
+      <xdr:rowOff>138600</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -1828,10 +1926,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="15546600" y="4287240"/>
-          <a:ext cx="1877400" cy="891360"/>
-          <a:chOff x="15546600" y="4287240"/>
-          <a:chExt cx="1877400" cy="891360"/>
+          <a:off x="15546600" y="4287600"/>
+          <a:ext cx="1876320" cy="890280"/>
+          <a:chOff x="15546600" y="4287600"/>
+          <a:chExt cx="1876320" cy="890280"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
@@ -1841,8 +1939,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="1649400">
-            <a:off x="15651720" y="4439880"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="15651720" y="4439520"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1865,7 +1963,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1874,13 +1976,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1895,8 +1995,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19608000">
-            <a:off x="16641360" y="4419360"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="16641000" y="4419360"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -1919,7 +2019,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -1928,13 +2032,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>12</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -1950,7 +2052,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="15763680" y="5080320"/>
-            <a:ext cx="1438200" cy="0"/>
+            <a:ext cx="1438200" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -1975,15 +2077,15 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>43560</xdr:colOff>
+      <xdr:colOff>51840</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>67320</xdr:rowOff>
+      <xdr:rowOff>128160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
-      <xdr:colOff>158760</xdr:colOff>
+      <xdr:colOff>167040</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>72720</xdr:rowOff>
+      <xdr:rowOff>133200</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -1992,10 +2094,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="17573760" y="3832200"/>
-          <a:ext cx="818280" cy="1740960"/>
-          <a:chOff x="17573760" y="3832200"/>
-          <a:chExt cx="818280" cy="1740960"/>
+          <a:off x="17582040" y="3893040"/>
+          <a:ext cx="817920" cy="1740960"/>
+          <a:chOff x="17582040" y="3893040"/>
+          <a:chExt cx="817920" cy="1740960"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
@@ -2005,8 +2107,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="16200000">
-            <a:off x="17550000" y="4929840"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="17558280" y="4991040"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -2029,7 +2131,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -2038,13 +2144,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -2059,8 +2163,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="16200000">
-            <a:off x="17748720" y="3910320"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="17757000" y="3971520"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -2083,7 +2187,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -2092,13 +2200,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>12</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -2113,7 +2219,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipH="1">
-            <a:off x="18194400" y="3832200"/>
+            <a:off x="18202680" y="3893040"/>
             <a:ext cx="19800" cy="1644840"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2139,15 +2245,15 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>301680</xdr:colOff>
+      <xdr:colOff>306720</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>96840</xdr:rowOff>
+      <xdr:rowOff>92160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>392760</xdr:colOff>
+      <xdr:colOff>397440</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>35640</xdr:rowOff>
+      <xdr:rowOff>30960</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2156,10 +2262,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="18178200" y="2052720"/>
-          <a:ext cx="1726920" cy="1716840"/>
-          <a:chOff x="18178200" y="2052720"/>
-          <a:chExt cx="1726920" cy="1716840"/>
+          <a:off x="18183240" y="2048040"/>
+          <a:ext cx="1726920" cy="1716480"/>
+          <a:chOff x="18183240" y="2048040"/>
+          <a:chExt cx="1726920" cy="1716480"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
@@ -2169,8 +2275,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="18699000">
-            <a:off x="18297720" y="2933280"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="18302760" y="2928240"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -2193,7 +2299,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -2202,13 +2312,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -2223,8 +2331,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="18699000">
-            <a:off x="19035000" y="2198160"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="19040040" y="2193120"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -2247,7 +2355,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -2256,13 +2368,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>12</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -2277,7 +2387,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipV="1">
-            <a:off x="18577080" y="2373480"/>
+            <a:off x="18582120" y="2368440"/>
             <a:ext cx="1328040" cy="1396080"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2311,7 +2421,7 @@
       <xdr:col>24</xdr:col>
       <xdr:colOff>642600</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>161640</xdr:rowOff>
+      <xdr:rowOff>161280</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2321,9 +2431,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="18489240" y="543960"/>
-          <a:ext cx="1660680" cy="1405800"/>
+          <a:ext cx="1660680" cy="1405440"/>
           <a:chOff x="18489240" y="543960"/>
-          <a:chExt cx="1660680" cy="1405800"/>
+          <a:chExt cx="1660680" cy="1405440"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
@@ -2334,7 +2444,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="18489240" y="543960"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -2357,7 +2467,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -2366,13 +2480,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -2388,7 +2500,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="18517680" y="1330200"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -2411,7 +2523,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -2420,13 +2536,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>12</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -2442,7 +2556,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="18613080" y="1198080"/>
-            <a:ext cx="1438200" cy="0"/>
+            <a:ext cx="1438200" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -2469,7 +2583,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="18711720" y="1935720"/>
-            <a:ext cx="1438200" cy="0"/>
+            <a:ext cx="1438200" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -2494,15 +2608,15 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>595080</xdr:colOff>
+      <xdr:colOff>573480</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>47160</xdr:rowOff>
+      <xdr:rowOff>68760</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>207720</xdr:colOff>
+      <xdr:colOff>186120</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>104040</xdr:rowOff>
+      <xdr:rowOff>125640</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2511,9 +2625,9 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="16872840" y="1651320"/>
+          <a:off x="16851240" y="1672920"/>
           <a:ext cx="381960" cy="425160"/>
-          <a:chOff x="16872840" y="1651320"/>
+          <a:chOff x="16851240" y="1672920"/>
           <a:chExt cx="381960" cy="425160"/>
         </a:xfrm>
       </xdr:grpSpPr>
@@ -2524,7 +2638,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="16872840" y="1651320"/>
+            <a:off x="16851240" y="1672920"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2551,7 +2665,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipH="1">
-            <a:off x="16872840" y="1651320"/>
+            <a:off x="16851240" y="1672920"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2577,15 +2691,15 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>213120</xdr:colOff>
+      <xdr:colOff>191520</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>59400</xdr:rowOff>
+      <xdr:rowOff>81000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>638280</xdr:colOff>
+      <xdr:colOff>616680</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>116280</xdr:rowOff>
+      <xdr:rowOff>137880</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2594,9 +2708,9 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="16490880" y="2638800"/>
+          <a:off x="16469280" y="2660400"/>
           <a:ext cx="381960" cy="425160"/>
-          <a:chOff x="16490880" y="2638800"/>
+          <a:chOff x="16469280" y="2660400"/>
           <a:chExt cx="381960" cy="425160"/>
         </a:xfrm>
       </xdr:grpSpPr>
@@ -2607,7 +2721,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="16490880" y="2638800"/>
+            <a:off x="16469280" y="2660400"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2634,7 +2748,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipH="1">
-            <a:off x="16490880" y="2638800"/>
+            <a:off x="16469280" y="2660400"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2659,16 +2773,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>3960</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>795240</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>134640</xdr:rowOff>
+      <xdr:rowOff>156240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>429120</xdr:colOff>
+      <xdr:colOff>407520</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>29160</xdr:rowOff>
+      <xdr:rowOff>50760</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2677,9 +2791,9 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="16281720" y="3526920"/>
+          <a:off x="16260120" y="3548520"/>
           <a:ext cx="381960" cy="425160"/>
-          <a:chOff x="16281720" y="3526920"/>
+          <a:chOff x="16260120" y="3548520"/>
           <a:chExt cx="381960" cy="425160"/>
         </a:xfrm>
       </xdr:grpSpPr>
@@ -2690,7 +2804,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="16281720" y="3526920"/>
+            <a:off x="16260120" y="3548520"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2717,7 +2831,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipH="1">
-            <a:off x="16281720" y="3526920"/>
+            <a:off x="16260120" y="3548520"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2743,15 +2857,15 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>792000</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>159480</xdr:rowOff>
+      <xdr:colOff>770400</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>18360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>404280</xdr:colOff>
+      <xdr:colOff>382680</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>53640</xdr:rowOff>
+      <xdr:rowOff>75240</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2760,9 +2874,9 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="16256880" y="4527000"/>
+          <a:off x="16235280" y="4548600"/>
           <a:ext cx="381960" cy="425160"/>
-          <a:chOff x="16256880" y="4527000"/>
+          <a:chOff x="16235280" y="4548600"/>
           <a:chExt cx="381960" cy="425160"/>
         </a:xfrm>
       </xdr:grpSpPr>
@@ -2773,7 +2887,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="16256880" y="4527000"/>
+            <a:off x="16235280" y="4548600"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2800,7 +2914,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipH="1">
-            <a:off x="16256880" y="4527000"/>
+            <a:off x="16235280" y="4548600"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2825,16 +2939,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>16200</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>33480</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>623160</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>156240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>441360</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>90360</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>235440</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>50400</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2843,9 +2957,9 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="18732240" y="2612880"/>
+          <a:off x="17713440" y="4523760"/>
           <a:ext cx="381960" cy="425160"/>
-          <a:chOff x="18732240" y="2612880"/>
+          <a:chOff x="17713440" y="4523760"/>
           <a:chExt cx="381960" cy="425160"/>
         </a:xfrm>
       </xdr:grpSpPr>
@@ -2856,7 +2970,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="18732240" y="2612880"/>
+            <a:off x="17713440" y="4523760"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2883,7 +2997,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipH="1">
-            <a:off x="18732240" y="2612880"/>
+            <a:off x="17713440" y="4523760"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2908,16 +3022,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>644760</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>134640</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>401040</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>106200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>257040</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>28800</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>13320</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>360</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2926,9 +3040,9 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="17735040" y="4502160"/>
+          <a:off x="19117080" y="1059840"/>
           <a:ext cx="381960" cy="425160"/>
-          <a:chOff x="17735040" y="4502160"/>
+          <a:chOff x="19117080" y="1059840"/>
           <a:chExt cx="381960" cy="425160"/>
         </a:xfrm>
       </xdr:grpSpPr>
@@ -2939,7 +3053,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="17735040" y="4502160"/>
+            <a:off x="19117080" y="1059840"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -2966,90 +3080,7 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm flipH="1">
-            <a:off x="17735040" y="4502160"/>
-            <a:ext cx="381960" cy="425160"/>
-          </a:xfrm>
-          <a:prstGeom prst="line">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:ln w="36720">
-            <a:solidFill>
-              <a:srgbClr val="FF4000"/>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="0"/>
-          <a:fillRef idx="0"/>
-          <a:effectRef idx="0"/>
-          <a:fontRef idx="minor"/>
-        </xdr:style>
-      </xdr:sp>
-    </xdr:grpSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>422640</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>84600</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>34920</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>141480</xdr:rowOff>
-    </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="61" name=""/>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
-        <a:xfrm>
-          <a:off x="19138680" y="1038240"/>
-          <a:ext cx="381960" cy="425160"/>
-          <a:chOff x="19138680" y="1038240"/>
-          <a:chExt cx="381960" cy="425160"/>
-        </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="62" name="Line 3"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="19138680" y="1038240"/>
-            <a:ext cx="381960" cy="425160"/>
-          </a:xfrm>
-          <a:prstGeom prst="line">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:ln w="36720">
-            <a:solidFill>
-              <a:srgbClr val="FF4000"/>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="0"/>
-          <a:fillRef idx="0"/>
-          <a:effectRef idx="0"/>
-          <a:fontRef idx="minor"/>
-        </xdr:style>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="63" name="Line 4"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm flipH="1">
-            <a:off x="19138680" y="1038240"/>
+            <a:off x="19117080" y="1059840"/>
             <a:ext cx="381960" cy="425160"/>
           </a:xfrm>
           <a:prstGeom prst="line">
@@ -3081,19 +3112,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>768240</xdr:colOff>
+      <xdr:colOff>767880</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>154800</xdr:rowOff>
+      <xdr:rowOff>154440</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="64" name="Text Frame 3"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvPr id="61" name="Text Frame 3"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="7320960" y="2382840"/>
-          <a:ext cx="1575360" cy="210240"/>
+          <a:ext cx="1575000" cy="209880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3103,11 +3134,22 @@
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -3149,45 +3191,45 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>178560</xdr:colOff>
+      <xdr:colOff>178200</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>83520</xdr:rowOff>
+      <xdr:rowOff>144000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="65" name=""/>
+        <xdr:cNvPr id="62" name=""/>
         <xdr:cNvGrpSpPr/>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="8840880" y="1374480"/>
-          <a:ext cx="3529800" cy="1960200"/>
+          <a:ext cx="3529440" cy="2020680"/>
           <a:chOff x="8840880" y="1374480"/>
-          <a:chExt cx="3529800" cy="1960200"/>
+          <a:chExt cx="3529440" cy="2020680"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:grpSp>
         <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="66" name=""/>
+          <xdr:cNvPr id="63" name=""/>
           <xdr:cNvGrpSpPr/>
         </xdr:nvGrpSpPr>
         <xdr:grpSpPr>
           <a:xfrm>
             <a:off x="8840880" y="1374480"/>
-            <a:ext cx="2381760" cy="1960200"/>
+            <a:ext cx="2380680" cy="1960200"/>
             <a:chOff x="8840880" y="1374480"/>
-            <a:chExt cx="2381760" cy="1960200"/>
+            <a:chExt cx="2380680" cy="1960200"/>
           </a:xfrm>
         </xdr:grpSpPr>
         <xdr:sp>
           <xdr:nvSpPr>
-            <xdr:cNvPr id="67" name="Shape 15"/>
+            <xdr:cNvPr id="64" name="Shape 15"/>
             <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm rot="19800000">
-              <a:off x="8951040" y="2589840"/>
-              <a:ext cx="667080" cy="619560"/>
+              <a:off x="8950680" y="2589840"/>
+              <a:ext cx="666720" cy="619200"/>
             </a:xfrm>
             <a:prstGeom prst="ellipse">
               <a:avLst/>
@@ -3210,7 +3252,11 @@
               <a:noAutofit/>
             </a:bodyPr>
             <a:p>
-              <a:pPr algn="ctr"/>
+              <a:pPr algn="ctr">
+                <a:lnSpc>
+                  <a:spcPct val="100000"/>
+                </a:lnSpc>
+              </a:pPr>
               <a:r>
                 <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                   <a:solidFill>
@@ -3219,13 +3265,11 @@
                   <a:effectLst/>
                   <a:uFillTx/>
                   <a:latin typeface="Times New Roman"/>
+                  <a:ea typeface="DejaVu Sans"/>
                 </a:rPr>
                 <a:t>8</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="00F4FF"/>
-                </a:solidFill>
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
@@ -3235,7 +3279,7 @@
         </xdr:sp>
         <xdr:sp>
           <xdr:nvSpPr>
-            <xdr:cNvPr id="68" name="Horizontal line 10"/>
+            <xdr:cNvPr id="65" name="Horizontal line 10"/>
             <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -3262,13 +3306,13 @@
         </xdr:sp>
         <xdr:sp>
           <xdr:nvSpPr>
-            <xdr:cNvPr id="69" name="Shape 20"/>
+            <xdr:cNvPr id="66" name="Shape 20"/>
             <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm rot="19800000">
               <a:off x="9603720" y="2351880"/>
-              <a:ext cx="775800" cy="287640"/>
+              <a:ext cx="775440" cy="287280"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3291,7 +3335,11 @@
               <a:noAutofit/>
             </a:bodyPr>
             <a:p>
-              <a:pPr algn="ctr"/>
+              <a:pPr algn="ctr">
+                <a:lnSpc>
+                  <a:spcPct val="100000"/>
+                </a:lnSpc>
+              </a:pPr>
               <a:r>
                 <a:rPr lang="en-US" sz="1800" b="0" u="none" strike="noStrike">
                   <a:solidFill>
@@ -3300,13 +3348,11 @@
                   <a:effectLst/>
                   <a:uFillTx/>
                   <a:latin typeface="Times New Roman"/>
+                  <a:ea typeface="DejaVu Sans"/>
                 </a:rPr>
                 <a:t>PPK</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1800" b="0" u="none" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="00F4FF"/>
-                </a:solidFill>
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
@@ -3316,13 +3362,13 @@
         </xdr:sp>
         <xdr:sp>
           <xdr:nvSpPr>
-            <xdr:cNvPr id="70" name="Shape 21"/>
+            <xdr:cNvPr id="67" name="Shape 21"/>
             <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm rot="19800000">
-              <a:off x="9471600" y="1999440"/>
-              <a:ext cx="1305360" cy="837720"/>
+              <a:off x="9471240" y="1999080"/>
+              <a:ext cx="1305000" cy="837360"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3344,13 +3390,13 @@
         </xdr:sp>
         <xdr:sp>
           <xdr:nvSpPr>
-            <xdr:cNvPr id="71" name="Text Frame 9"/>
-            <xdr:cNvSpPr txBox="1"/>
+            <xdr:cNvPr id="68" name="Text Frame 9"/>
+            <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm rot="19800000">
               <a:off x="9306360" y="1759680"/>
-              <a:ext cx="1662840" cy="450360"/>
+              <a:ext cx="1662480" cy="450000"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3360,11 +3406,22 @@
               <a:noFill/>
             </a:ln>
           </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0"/>
+            <a:fillRef idx="0"/>
+            <a:effectRef idx="0"/>
+            <a:fontRef idx="minor"/>
+          </xdr:style>
           <xdr:txBody>
             <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
               <a:noAutofit/>
             </a:bodyPr>
             <a:p>
+              <a:pPr>
+                <a:lnSpc>
+                  <a:spcPct val="100000"/>
+                </a:lnSpc>
+              </a:pPr>
               <a:r>
                 <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
                   <a:solidFill>
@@ -3386,13 +3443,13 @@
         </xdr:sp>
         <xdr:sp>
           <xdr:nvSpPr>
-            <xdr:cNvPr id="72" name="Text Frame 10"/>
-            <xdr:cNvSpPr txBox="1"/>
+            <xdr:cNvPr id="69" name="Text Frame 10"/>
+            <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm rot="19800000">
-              <a:off x="10746000" y="1818360"/>
-              <a:ext cx="406440" cy="388080"/>
+              <a:off x="10745640" y="1818000"/>
+              <a:ext cx="406080" cy="387720"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3402,11 +3459,22 @@
               <a:noFill/>
             </a:ln>
           </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0"/>
+            <a:fillRef idx="0"/>
+            <a:effectRef idx="0"/>
+            <a:fontRef idx="minor"/>
+          </xdr:style>
           <xdr:txBody>
             <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
               <a:noAutofit/>
             </a:bodyPr>
             <a:p>
+              <a:pPr>
+                <a:lnSpc>
+                  <a:spcPct val="100000"/>
+                </a:lnSpc>
+              </a:pPr>
               <a:r>
                 <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
                   <a:solidFill>
@@ -3429,13 +3497,13 @@
       </xdr:grpSp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="73" name="Horizontal line 11"/>
+          <xdr:cNvPr id="70" name="Horizontal line 11"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="9051840" y="3238560"/>
-            <a:ext cx="2512080" cy="0"/>
+            <a:ext cx="2512080" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -3455,13 +3523,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="74" name="Elliptical arc 1"/>
+          <xdr:cNvPr id="71" name="Elliptical arc 1"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="18091200">
             <a:off x="10406160" y="2658240"/>
-            <a:ext cx="696600" cy="577800"/>
+            <a:ext cx="696240" cy="577440"/>
           </a:xfrm>
           <a:prstGeom prst="arc">
             <a:avLst>
@@ -3477,16 +3545,22 @@
             <a:tailEnd len="med" type="triangle" w="med"/>
           </a:ln>
         </xdr:spPr>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="75" name="Text Frame 4"/>
-          <xdr:cNvSpPr txBox="1"/>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="72" name="Text Frame 4"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="11120400" y="2827080"/>
-            <a:ext cx="1250280" cy="355320"/>
+            <a:ext cx="1249920" cy="354960"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3496,11 +3570,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -3519,6 +3604,11 @@
             </a:endParaRPr>
           </a:p>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -3550,19 +3640,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>748080</xdr:colOff>
+      <xdr:colOff>747720</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>18000</xdr:rowOff>
+      <xdr:rowOff>17640</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="76" name="Text Frame 11"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvPr id="73" name="Text Frame 11"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1325520" y="6699240"/>
-          <a:ext cx="2673720" cy="633960"/>
+          <a:ext cx="2673360" cy="633600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3575,12 +3665,22 @@
           <a:round/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="18000" tIns="18000" rIns="18000" bIns="18000" anchor="ctr">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr algn="ctr">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="2000" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -3593,9 +3693,6 @@
             <a:t>公差配對規則</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="2000" b="0" u="none" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="00F4FF"/>
-            </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
@@ -3610,36 +3707,36 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>605520</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>20520</xdr:rowOff>
+      <xdr:rowOff>20160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>333720</xdr:colOff>
+      <xdr:colOff>333360</xdr:colOff>
       <xdr:row>61</xdr:row>
-      <xdr:rowOff>64440</xdr:rowOff>
+      <xdr:rowOff>124920</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="77" name=""/>
+        <xdr:cNvPr id="74" name=""/>
         <xdr:cNvGrpSpPr/>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1418400" y="7335720"/>
-          <a:ext cx="3792240" cy="2644920"/>
-          <a:chOff x="1418400" y="7335720"/>
-          <a:chExt cx="3792240" cy="2644920"/>
+          <a:off x="1418400" y="7335360"/>
+          <a:ext cx="3791880" cy="2705760"/>
+          <a:chOff x="1418400" y="7335360"/>
+          <a:chExt cx="3791880" cy="2705760"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="78" name="Shape 15"/>
+          <xdr:cNvPr id="75" name="Shape 15"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19800000">
-            <a:off x="1528560" y="9235800"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="1528200" y="9235800"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -3662,7 +3759,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -3671,13 +3772,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -3687,7 +3786,7 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="79" name="Horizontal line 10"/>
+          <xdr:cNvPr id="76" name="Horizontal line 10"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
@@ -3714,13 +3813,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="80" name="Shape 21"/>
+          <xdr:cNvPr id="77" name="Shape 21"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19800000">
-            <a:off x="1971000" y="8353800"/>
-            <a:ext cx="2471400" cy="837720"/>
+            <a:off x="1970640" y="8353800"/>
+            <a:ext cx="2471040" cy="837360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3742,13 +3841,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="81" name="Text Frame 9"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="78" name="Text Frame 9"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19800000">
-            <a:off x="1864080" y="8331480"/>
-            <a:ext cx="1959480" cy="450360"/>
+            <a:off x="1863720" y="8331480"/>
+            <a:ext cx="1959120" cy="450000"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3758,11 +3857,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -3784,13 +3894,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="82" name="Text Frame 10"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="79" name="Text Frame 10"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="3600600">
-            <a:off x="3567600" y="8199720"/>
-            <a:ext cx="2093040" cy="168840"/>
+            <a:off x="3567600" y="8199360"/>
+            <a:ext cx="2092680" cy="168480"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3800,11 +3910,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1200" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -3826,13 +3947,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="83" name="Horizontal line 11"/>
+          <xdr:cNvPr id="80" name="Horizontal line 11"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="1629360" y="9884520"/>
-            <a:ext cx="2512080" cy="0"/>
+            <a:ext cx="2512080" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -3852,13 +3973,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="84" name="Elliptical arc 1"/>
+          <xdr:cNvPr id="81" name="Elliptical arc 1"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="18091200">
             <a:off x="2983680" y="9304200"/>
-            <a:ext cx="696600" cy="577800"/>
+            <a:ext cx="696240" cy="577440"/>
           </a:xfrm>
           <a:prstGeom prst="arc">
             <a:avLst>
@@ -3874,16 +3995,22 @@
             <a:tailEnd len="med" type="triangle" w="med"/>
           </a:ln>
         </xdr:spPr>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="85" name="Text Frame 4"/>
-          <xdr:cNvSpPr txBox="1"/>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="82" name="Text Frame 4"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="3661920" y="9545040"/>
-            <a:ext cx="1250280" cy="253080"/>
+            <a:ext cx="1249920" cy="252720"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3893,11 +4020,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -3919,13 +4057,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="86" name="Text Frame 12"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="83" name="Text Frame 12"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19840800">
-            <a:off x="2333520" y="8582040"/>
-            <a:ext cx="2100600" cy="675720"/>
+            <a:off x="2333160" y="8582040"/>
+            <a:ext cx="2100240" cy="675360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3935,11 +4073,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -3952,9 +4101,6 @@
               <a:t>214.50±0.15</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="FFFF00"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -3968,38 +4114,38 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>11160</xdr:colOff>
+      <xdr:colOff>10800</xdr:colOff>
       <xdr:row>47</xdr:row>
       <xdr:rowOff>105840</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>608400</xdr:colOff>
+      <xdr:colOff>608040</xdr:colOff>
       <xdr:row>61</xdr:row>
-      <xdr:rowOff>50040</xdr:rowOff>
+      <xdr:rowOff>49320</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="87" name=""/>
+        <xdr:cNvPr id="84" name=""/>
         <xdr:cNvGrpSpPr/>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="5700600" y="7746120"/>
-          <a:ext cx="3848760" cy="2220120"/>
-          <a:chOff x="5700600" y="7746120"/>
-          <a:chExt cx="3848760" cy="2220120"/>
+          <a:off x="5700240" y="7746120"/>
+          <a:ext cx="3848760" cy="2219400"/>
+          <a:chOff x="5700240" y="7746120"/>
+          <a:chExt cx="3848760" cy="2219400"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="88" name="Shape 17"/>
+          <xdr:cNvPr id="85" name="Shape 17"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19800000">
-            <a:off x="8049600" y="7871040"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:off x="8049240" y="7871040"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -4022,7 +4168,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4031,13 +4181,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -4047,7 +4195,7 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="89" name="Horizontal line 12"/>
+          <xdr:cNvPr id="86" name="Horizontal line 12"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
@@ -4074,13 +4222,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="90" name="Shape 18"/>
+          <xdr:cNvPr id="87" name="Shape 18"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19800000">
-            <a:off x="5744160" y="8566560"/>
-            <a:ext cx="2471400" cy="837720"/>
+            <a:off x="5743800" y="8566560"/>
+            <a:ext cx="2471040" cy="837360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4102,13 +4250,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="91" name="Horizontal line 13"/>
+          <xdr:cNvPr id="88" name="Horizontal line 13"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="6266520" y="9701280"/>
-            <a:ext cx="2512080" cy="0"/>
+            <a:ext cx="2512080" cy="360"/>
           </a:xfrm>
           <a:prstGeom prst="line">
             <a:avLst/>
@@ -4128,13 +4276,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="92" name="Elliptical arc 2"/>
+          <xdr:cNvPr id="89" name="Elliptical arc 2"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="18091200">
             <a:off x="7620840" y="9120960"/>
-            <a:ext cx="696600" cy="577800"/>
+            <a:ext cx="696240" cy="577440"/>
           </a:xfrm>
           <a:prstGeom prst="arc">
             <a:avLst>
@@ -4150,16 +4298,22 @@
             <a:tailEnd len="med" type="triangle" w="med"/>
           </a:ln>
         </xdr:spPr>
-      </xdr:sp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="93" name="Text Frame 15"/>
-          <xdr:cNvSpPr txBox="1"/>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
+      </xdr:sp>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="90" name="Text Frame 15"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="8299080" y="9361800"/>
-            <a:ext cx="1250280" cy="253080"/>
+            <a:ext cx="1249920" cy="252720"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4169,11 +4323,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="zh-CN" sz="1200" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4195,13 +4360,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="94" name="Text Frame 16"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="91" name="Text Frame 16"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="19840800">
-            <a:off x="6106680" y="8794800"/>
-            <a:ext cx="2100600" cy="675720"/>
+            <a:off x="6106320" y="8794800"/>
+            <a:ext cx="2100240" cy="675360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4211,11 +4376,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4228,9 +4404,6 @@
               <a:t>214.50±0.15</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="FFFF00"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -4246,36 +4419,36 @@
       <xdr:col>13</xdr:col>
       <xdr:colOff>341280</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>133920</xdr:rowOff>
+      <xdr:rowOff>134280</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>700560</xdr:colOff>
+      <xdr:colOff>699840</xdr:colOff>
       <xdr:row>63</xdr:row>
-      <xdr:rowOff>23400</xdr:rowOff>
+      <xdr:rowOff>23040</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="95" name=""/>
+        <xdr:cNvPr id="92" name=""/>
         <xdr:cNvGrpSpPr/>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10907640" y="6148800"/>
-          <a:ext cx="2797560" cy="4115880"/>
-          <a:chOff x="10907640" y="6148800"/>
-          <a:chExt cx="2797560" cy="4115880"/>
+          <a:off x="10907640" y="6149160"/>
+          <a:ext cx="2796840" cy="4115160"/>
+          <a:chOff x="10907640" y="6149160"/>
+          <a:chExt cx="2796840" cy="4115160"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="96" name="Shape 19"/>
+          <xdr:cNvPr id="93" name="Shape 19"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="11603160" y="8545320"/>
-            <a:ext cx="667080" cy="619560"/>
+            <a:ext cx="666720" cy="619200"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -4298,7 +4471,11 @@
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
-            <a:pPr algn="ctr"/>
+            <a:pPr algn="ctr">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4307,13 +4484,11 @@
                 <a:effectLst/>
                 <a:uFillTx/>
                 <a:latin typeface="Times New Roman"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>8</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="00F4FF"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -4323,13 +4498,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="97" name="Shape 22"/>
+          <xdr:cNvPr id="94" name="Shape 22"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="10907640" y="7926480"/>
-            <a:ext cx="2044080" cy="1900800"/>
+            <a:ext cx="2043720" cy="1900440"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4352,13 +4527,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="98" name="Text Frame 13"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="95" name="Text Frame 13"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="40800">
-            <a:off x="11225160" y="9241200"/>
-            <a:ext cx="2100600" cy="675720"/>
+            <a:off x="11224800" y="9240840"/>
+            <a:ext cx="2100240" cy="675360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4368,11 +4543,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4385,9 +4571,6 @@
               <a:t>214.50±0.15</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="FFFF00"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -4397,13 +4580,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="99" name="Text Frame 14"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="96" name="Text Frame 14"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="16240800">
-            <a:off x="10461600" y="6865200"/>
-            <a:ext cx="2100600" cy="675720"/>
+            <a:off x="10461240" y="6865560"/>
+            <a:ext cx="2100240" cy="675360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4413,11 +4596,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4430,9 +4624,6 @@
               <a:t>214.50±0.15</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="FFFF00"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -4442,13 +4633,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="100" name="Text Frame 17"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="97" name="Text Frame 17"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="18040800">
             <a:off x="11828160" y="7102440"/>
-            <a:ext cx="2100600" cy="675720"/>
+            <a:ext cx="2100240" cy="675360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4458,11 +4649,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4475,9 +4677,6 @@
               <a:t>214.50±0.15</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="FFFF00"/>
-              </a:solidFill>
               <a:effectLst/>
               <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
@@ -4487,13 +4686,13 @@
       </xdr:sp>
       <xdr:sp>
         <xdr:nvSpPr>
-          <xdr:cNvPr id="101" name="Text Frame 18"/>
-          <xdr:cNvSpPr txBox="1"/>
+          <xdr:cNvPr id="98" name="Text Frame 18"/>
+          <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="11143080" y="9876960"/>
-            <a:ext cx="1638000" cy="387720"/>
+            <a:ext cx="1637640" cy="387360"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -4503,11 +4702,22 @@
             <a:noFill/>
           </a:ln>
         </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0"/>
+          <a:fillRef idx="0"/>
+          <a:effectRef idx="0"/>
+          <a:fontRef idx="minor"/>
+        </xdr:style>
         <xdr:txBody>
           <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
             <a:noAutofit/>
           </a:bodyPr>
           <a:p>
+            <a:pPr>
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+            </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1400" b="0" u="none" strike="noStrike">
                 <a:solidFill>
@@ -4529,7 +4739,7 @@
       </xdr:sp>
       <xdr:grpSp>
         <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="102" name=""/>
+          <xdr:cNvPr id="99" name=""/>
           <xdr:cNvGrpSpPr/>
         </xdr:nvGrpSpPr>
         <xdr:grpSpPr>
@@ -4542,12 +4752,80 @@
         </xdr:grpSpPr>
         <xdr:sp>
           <xdr:nvSpPr>
+            <xdr:cNvPr id="100" name="Line 3"/>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="11193120" y="7439400"/>
+              <a:ext cx="381960" cy="425160"/>
+            </a:xfrm>
+            <a:prstGeom prst="line">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:ln w="36720">
+              <a:solidFill>
+                <a:srgbClr val="FF4000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0"/>
+            <a:fillRef idx="0"/>
+            <a:effectRef idx="0"/>
+            <a:fontRef idx="minor"/>
+          </xdr:style>
+        </xdr:sp>
+        <xdr:sp>
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="101" name="Line 4"/>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm flipH="1">
+              <a:off x="11193120" y="7439400"/>
+              <a:ext cx="381960" cy="425160"/>
+            </a:xfrm>
+            <a:prstGeom prst="line">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:ln w="36720">
+              <a:solidFill>
+                <a:srgbClr val="FF4000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0"/>
+            <a:fillRef idx="0"/>
+            <a:effectRef idx="0"/>
+            <a:fontRef idx="minor"/>
+          </xdr:style>
+        </xdr:sp>
+      </xdr:grpSp>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="102" name=""/>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="12424680" y="7414560"/>
+            <a:ext cx="381960" cy="425160"/>
+            <a:chOff x="12424680" y="7414560"/>
+            <a:chExt cx="381960" cy="425160"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:sp>
+          <xdr:nvSpPr>
             <xdr:cNvPr id="103" name="Line 3"/>
             <xdr:cNvSpPr/>
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="11193120" y="7439400"/>
+              <a:off x="12424680" y="7414560"/>
               <a:ext cx="381960" cy="425160"/>
             </a:xfrm>
             <a:prstGeom prst="line">
@@ -4574,7 +4852,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm flipH="1">
-              <a:off x="11193120" y="7439400"/>
+              <a:off x="12424680" y="7414560"/>
               <a:ext cx="381960" cy="425160"/>
             </a:xfrm>
             <a:prstGeom prst="line">
@@ -4595,83 +4873,15 @@
           </xdr:style>
         </xdr:sp>
       </xdr:grpSp>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="105" name=""/>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="12424680" y="7414560"/>
-            <a:ext cx="381960" cy="425160"/>
-            <a:chOff x="12424680" y="7414560"/>
-            <a:chExt cx="381960" cy="425160"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:sp>
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="106" name="Line 3"/>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="12424680" y="7414560"/>
-              <a:ext cx="381960" cy="425160"/>
-            </a:xfrm>
-            <a:prstGeom prst="line">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:ln w="36720">
-              <a:solidFill>
-                <a:srgbClr val="FF4000"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0"/>
-            <a:fillRef idx="0"/>
-            <a:effectRef idx="0"/>
-            <a:fontRef idx="minor"/>
-          </xdr:style>
-        </xdr:sp>
-        <xdr:sp>
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="107" name="Line 4"/>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm flipH="1">
-              <a:off x="12424680" y="7414560"/>
-              <a:ext cx="381960" cy="425160"/>
-            </a:xfrm>
-            <a:prstGeom prst="line">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:ln w="36720">
-              <a:solidFill>
-                <a:srgbClr val="FF4000"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0"/>
-            <a:fillRef idx="0"/>
-            <a:effectRef idx="0"/>
-            <a:fontRef idx="minor"/>
-          </xdr:style>
-        </xdr:sp>
-      </xdr:grpSp>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="108" name="Shape 23"/>
+      <xdr:sp>
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="105" name="Shape 23"/>
           <xdr:cNvSpPr/>
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="11779920" y="9240840"/>
-            <a:ext cx="369720" cy="369720"/>
+            <a:ext cx="369360" cy="369360"/>
           </a:xfrm>
           <a:prstGeom prst="ellipse">
             <a:avLst/>
@@ -4703,19 +4913,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
-      <xdr:colOff>668880</xdr:colOff>
+      <xdr:colOff>668520</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>95040</xdr:rowOff>
+      <xdr:rowOff>94680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="109" name="Text Frame 19"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvPr id="106" name="Text Frame 19"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="19848240" y="4280760"/>
-          <a:ext cx="3579120" cy="1341360"/>
+          <a:ext cx="3578760" cy="1341000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4725,11 +4935,22 @@
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -4759,6 +4980,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -4777,6 +5003,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -4795,6 +5026,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="2100" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -4825,19 +5061,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>530280</xdr:colOff>
+      <xdr:colOff>529920</xdr:colOff>
       <xdr:row>71</xdr:row>
-      <xdr:rowOff>60840</xdr:rowOff>
+      <xdr:rowOff>60480</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="110" name="Shape 24"/>
+        <xdr:cNvPr id="107" name="Shape 24"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="949680" y="6471000"/>
-          <a:ext cx="13398120" cy="5131440"/>
+          <a:ext cx="13397760" cy="5131080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4868,19 +5104,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>504000</xdr:colOff>
+      <xdr:colOff>503640</xdr:colOff>
       <xdr:row>70</xdr:row>
-      <xdr:rowOff>47520</xdr:rowOff>
+      <xdr:rowOff>47160</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="111" name="Text Frame 20"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvPr id="108" name="Text Frame 20"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1644480" y="10695240"/>
-          <a:ext cx="2923560" cy="731520"/>
+          <a:ext cx="2923200" cy="731160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4890,11 +5126,22 @@
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1600" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -4946,6 +5193,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1600" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -4976,19 +5228,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>163080</xdr:colOff>
+      <xdr:colOff>162720</xdr:colOff>
       <xdr:row>70</xdr:row>
-      <xdr:rowOff>47520</xdr:rowOff>
+      <xdr:rowOff>47160</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="112" name="Text Frame 21"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvPr id="109" name="Text Frame 21"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6180480" y="10695240"/>
-          <a:ext cx="2923560" cy="731520"/>
+          <a:ext cx="2923200" cy="731160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4998,11 +5250,22 @@
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1600" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -5054,6 +5317,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1600" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -5084,19 +5352,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>150120</xdr:colOff>
+      <xdr:colOff>149760</xdr:colOff>
       <xdr:row>70</xdr:row>
-      <xdr:rowOff>47520</xdr:rowOff>
+      <xdr:rowOff>47160</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="113" name="Text Frame 22"/>
-        <xdr:cNvSpPr txBox="1"/>
+        <xdr:cNvPr id="110" name="Text Frame 22"/>
+        <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10585440" y="10695240"/>
-          <a:ext cx="3382200" cy="731520"/>
+          <a:ext cx="3381840" cy="731160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5106,11 +5374,22 @@
           <a:noFill/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
       <xdr:txBody>
         <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="zh-CN" sz="1600" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -5162,6 +5441,11 @@
           </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1600" b="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -5192,25 +5476,31 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>366840</xdr:colOff>
+      <xdr:colOff>366480</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>54000</xdr:rowOff>
+      <xdr:rowOff>53640</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="114" name="Polyline with 3 points 3"/>
+        <xdr:cNvPr id="111" name="Polyline with 3 points 3"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6187320" y="4226400"/>
-          <a:ext cx="4745880" cy="1191960"/>
+          <a:ext cx="4745520" cy="1191600"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
-          <a:gdLst/>
+          <a:gdLst>
+            <a:gd name="textAreaLeft" fmla="*/ 0 w 4745520"/>
+            <a:gd name="textAreaRight" fmla="*/ 4745880 w 4745520"/>
+            <a:gd name="textAreaTop" fmla="*/ 0 h 1191600"/>
+            <a:gd name="textAreaBottom" fmla="*/ 1191960 h 1191600"/>
+          </a:gdLst>
           <a:ahLst/>
-          <a:rect l="0" t="0" r="r" b="b"/>
+          <a:cxnLst/>
+          <a:rect l="textAreaLeft" t="textAreaTop" r="textAreaRight" b="textAreaBottom"/>
           <a:pathLst>
             <a:path fill="none" w="13183" h="3311">
               <a:moveTo>
@@ -5225,6 +5515,7 @@
             </a:path>
           </a:pathLst>
         </a:custGeom>
+        <a:noFill/>
         <a:ln cap="rnd" w="18360">
           <a:solidFill>
             <a:srgbClr val="FFD8CE"/>
@@ -5234,6 +5525,113 @@
           <a:tailEnd len="med" type="triangle" w="med"/>
         </a:ln>
       </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>116280</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>480960</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>129960</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="112" name="Shape 25"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17997840" y="2113200"/>
+          <a:ext cx="1990440" cy="1593000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln cap="rnd" w="0">
+          <a:solidFill>
+            <a:srgbClr val="FFD8CE"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>315000</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>146520</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>232200</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>113760</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="113" name="Text Frame 5"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19009440" y="3072600"/>
+          <a:ext cx="1542600" cy="455040"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="FFFF00"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
+              <a:latin typeface="Times New Roman"/>
+            </a:rPr>
+            <a:t>under test</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="2400" b="0" u="none" strike="noStrike">
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>

</xml_diff>